<commit_message>
fix(gm): register addtestitems as normal GM command and remove hardcoded toolbar button
</commit_message>
<xml_diff>
--- a/tables/datas/common/TbGmCommandDesc_new.xlsx
+++ b/tables/datas/common/TbGmCommandDesc_new.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,6 +591,23 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>addtestitems</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>添加测试道具</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>